<commit_message>
Rerun analyses, format tables
</commit_message>
<xml_diff>
--- a/plots/livlipid_betaglm_table.xlsx
+++ b/plots/livlipid_betaglm_table.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="61">
   <si>
     <t>common_name</t>
   </si>
@@ -95,15 +95,12 @@
     <t>14.3</t>
   </si>
   <si>
-    <t>13.9</t>
+    <t>13.3</t>
   </si>
   <si>
     <t>15.2</t>
   </si>
   <si>
-    <t>13.3</t>
-  </si>
-  <si>
     <t>13.1</t>
   </si>
   <si>
@@ -119,7 +116,7 @@
     <t>42.6</t>
   </si>
   <si>
-    <t>45.5</t>
+    <t>43.7</t>
   </si>
   <si>
     <t>50.4</t>
@@ -131,7 +128,7 @@
     <t>44.8</t>
   </si>
   <si>
-    <t>61.4</t>
+    <t>61.8</t>
   </si>
   <si>
     <t>71.8</t>
@@ -143,7 +140,7 @@
     <t>10.3</t>
   </si>
   <si>
-    <t>10.8</t>
+    <t>10.2</t>
   </si>
   <si>
     <t>11.3</t>
@@ -152,7 +149,7 @@
     <t xml:space="preserve"> 9.8</t>
   </si>
   <si>
-    <t>13.6</t>
+    <t>13.7</t>
   </si>
   <si>
     <t>14.6</t>
@@ -164,7 +161,7 @@
     <t>0.28</t>
   </si>
   <si>
-    <t>0.30</t>
+    <t>0.36</t>
   </si>
   <si>
     <t>0.17</t>
@@ -185,7 +182,7 @@
     <t>-0.008</t>
   </si>
   <si>
-    <t xml:space="preserve"> 0.005</t>
+    <t>-0.001</t>
   </si>
   <si>
     <t>-0.010</t>
@@ -303,16 +300,16 @@
         <v>25</v>
       </c>
       <c r="H2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="K2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3">
@@ -338,16 +335,16 @@
         <v>26</v>
       </c>
       <c r="H3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="K3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4">
@@ -364,25 +361,25 @@
         <v>23</v>
       </c>
       <c r="E4" t="n">
-        <v>-92.01</v>
+        <v>-87.65</v>
       </c>
       <c r="F4" t="n">
-        <v>34.95</v>
+        <v>39.31</v>
       </c>
       <c r="G4" t="s">
         <v>27</v>
       </c>
       <c r="H4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="K4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5">
@@ -408,16 +405,16 @@
         <v>28</v>
       </c>
       <c r="H5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6">
@@ -440,19 +437,19 @@
         <v>0.0</v>
       </c>
       <c r="G6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="K6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7">
@@ -475,19 +472,19 @@
         <v>26.28</v>
       </c>
       <c r="G7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="K7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8">
@@ -504,25 +501,25 @@
         <v>24</v>
       </c>
       <c r="E8" t="n">
-        <v>-74.99</v>
+        <v>-74.14</v>
       </c>
       <c r="F8" t="n">
-        <v>60.04</v>
+        <v>60.89</v>
       </c>
       <c r="G8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9">
@@ -545,19 +542,19 @@
         <v>71.19</v>
       </c>
       <c r="G9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="K9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>